<commit_message>
docs: README run instructions update, task plan tracking
README: migration-up gotcha for a stack already running, worker's dual
RAG+sim role, PDF Simulator testing walkthrough, completed the Other
Commands list, seeded-credential staleness caveat.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/EduAI_Task_Plan.WEEKLY.xlsx
+++ b/EduAI_Task_Plan.WEEKLY.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Weekly Summary" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Task Tracker'!$A$2:$F$89</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Task Tracker'!$A$2:$F$84</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="183">
   <si>
     <t>EduAI - Weekly Task Plan   |   Deadline 31 Aug 2026   |   Working days: Mon-Fri plus 2nd and 4th Saturdays.   Off: all Sundays, the 1st/3rd/5th Saturdays, and 15, 16, 23, 28, 29, 30 Aug.   |   All testing is scheduled last (27 and 31 Aug).</t>
   </si>
@@ -150,135 +150,126 @@
     <t>School onboarding - transactional and retry</t>
   </si>
   <si>
+    <t>Changed</t>
+  </si>
+  <si>
+    <t>13 Aug 2026: school, entitlements, auth user and profile are still separate writes with cleanup logic.</t>
+  </si>
+  <si>
+    <t>Entitlement limits and enforcement</t>
+  </si>
+  <si>
+    <t>13 Aug 2026: enforcement done (requireFeature + explicit ENTITLEMENTS_FAILURE_MODE). Seat/storage/AI limits not built.</t>
+  </si>
+  <si>
+    <t>Audit log viewer - filters and export</t>
+  </si>
+  <si>
+    <t>13 Aug 2026: filters by action/entity/actor/search + CSV export sharing the same query. /audit-log/actions supplies the vocabulary.</t>
+  </si>
+  <si>
+    <t>Cross-school lookup logging</t>
+  </si>
+  <si>
+    <t>13 Aug 2026: already shipped — student_directory.search is recorded with the query and result count.</t>
+  </si>
+  <si>
+    <t>Fri 14 Aug</t>
+  </si>
+  <si>
+    <t>School logo upload validation</t>
+  </si>
+  <si>
+    <t>13 Aug 2026: magic-byte sniffing (PNG/JPEG/WEBP) and declared MIME must match. Previously trusted client-supplied mimetype into a public bucket.</t>
+  </si>
+  <si>
+    <t>Pagination for schools and overview</t>
+  </si>
+  <si>
+    <t>13 Aug 2026: API paginated + searchable; overview counts moved to a SQL aggregate (was loading every user_profile). Pager UI on the Schools screen still to build.</t>
+  </si>
+  <si>
+    <t>3. Mail Providers (all modules)</t>
+  </si>
+  <si>
+    <t>Configure mail provider and templates</t>
+  </si>
+  <si>
+    <t>17 Aug 2026: SMTP transport + one template (school-admin welcome) exist. Remaining templates not built.</t>
+  </si>
+  <si>
+    <t>School onboarding welcome email</t>
+  </si>
+  <si>
+    <t>17 Aug 2026: already shipped — sendSchoolAdminWelcomeEmail fires on school creation and on adding an admin.</t>
+  </si>
+  <si>
+    <t>Week 2 (17-22 Aug)</t>
+  </si>
+  <si>
+    <t>Mon 17 Aug</t>
+  </si>
+  <si>
+    <t>Support ticket  - school admin</t>
+  </si>
+  <si>
+    <t>17 Aug 2026: not started.</t>
+  </si>
+  <si>
+    <t>Exam result and report notification</t>
+  </si>
+  <si>
     <t>Pending</t>
   </si>
   <si>
-    <t>13 Aug 2026: school, entitlements, auth user and profile are still separate writes with cleanup logic.</t>
-  </si>
-  <si>
-    <t>Entitlement limits and enforcement</t>
-  </si>
-  <si>
-    <t>13 Aug 2026: enforcement done (requireFeature + explicit ENTITLEMENTS_FAILURE_MODE). Seat/storage/AI limits not built.</t>
-  </si>
-  <si>
-    <t>Audit log viewer - filters and export</t>
-  </si>
-  <si>
-    <t>13 Aug 2026: filters by action/entity/actor/search + CSV export sharing the same query. /audit-log/actions supplies the vocabulary.</t>
-  </si>
-  <si>
-    <t>Cross-school lookup logging</t>
-  </si>
-  <si>
-    <t>13 Aug 2026: already shipped — student_directory.search is recorded with the query and result count.</t>
-  </si>
-  <si>
-    <t>Fri 14 Aug</t>
-  </si>
-  <si>
-    <t>School logo upload validation</t>
-  </si>
-  <si>
-    <t>13 Aug 2026: magic-byte sniffing (PNG/JPEG/WEBP) and declared MIME must match. Previously trusted client-supplied mimetype into a public bucket.</t>
-  </si>
-  <si>
-    <t>Pagination for schools and overview</t>
-  </si>
-  <si>
-    <t>13 Aug 2026: API paginated + searchable; overview counts moved to a SQL aggregate (was loading every user_profile). Pager UI on the Schools screen still to build.</t>
-  </si>
-  <si>
-    <t>3. Mail Providers (all modules)</t>
-  </si>
-  <si>
-    <t>Configure mail provider and templates</t>
+    <t>17 Aug 2026: not started. Result RELEASE control now exists, so a notification has a trigger to hang off.</t>
+  </si>
+  <si>
+    <t>Bounce and failure logging</t>
+  </si>
+  <si>
+    <t>17 Aug 2026: sendMail is fire-and-forget; failures are logged but not recorded per recipient.</t>
+  </si>
+  <si>
+    <t>4. Timetable and Lab</t>
+  </si>
+  <si>
+    <t>Conflict detection and clear messages</t>
+  </si>
+  <si>
+    <t>17 Aug 2026: already shipped — unique constraints on teacher/section/lab per period, mapped to plain-English messages, plus a lab seat-capacity warning.</t>
+  </si>
+  <si>
+    <t>Computer lab allocation</t>
+  </si>
+  <si>
+    <t>17 Aug 2026: already shipped — lab_id on timetable slots with capacity warning.</t>
+  </si>
+  <si>
+    <t>Link live session to timetable period</t>
+  </si>
+  <si>
+    <t>17 Aug 2026: live_sessions has no timetable_slot_id — sessions are not tied to a scheduled period.</t>
+  </si>
+  <si>
+    <t>Tue 18 Aug</t>
+  </si>
+  <si>
+    <t>Substitute teacher and rescheduling</t>
   </si>
   <si>
     <t>In progress</t>
   </si>
   <si>
-    <t>17 Aug 2026: SMTP transport + one template (school-admin welcome) exist. Remaining templates not built.</t>
-  </si>
-  <si>
-    <t>School onboarding welcome email</t>
-  </si>
-  <si>
-    <t>17 Aug 2026: already shipped — sendSchoolAdminWelcomeEmail fires on school creation and on adding an admin.</t>
-  </si>
-  <si>
-    <t>Week 2 (17-22 Aug)</t>
-  </si>
-  <si>
-    <t>Mon 17 Aug</t>
-  </si>
-  <si>
-    <t>Support ticket notification email</t>
-  </si>
-  <si>
-    <t>17 Aug 2026: not started.</t>
-  </si>
-  <si>
-    <t>Exam result and report notification</t>
-  </si>
-  <si>
-    <t>17 Aug 2026: not started. Result RELEASE control now exists, so a notification has a trigger to hang off.</t>
-  </si>
-  <si>
-    <t>Bounce and failure logging</t>
-  </si>
-  <si>
-    <t>17 Aug 2026: sendMail is fire-and-forget; failures are logged but not recorded per recipient.</t>
-  </si>
-  <si>
-    <t>4. Timetable and Lab</t>
-  </si>
-  <si>
-    <t>Conflict detection and clear messages</t>
-  </si>
-  <si>
-    <t>17 Aug 2026: already shipped — unique constraints on teacher/section/lab per period, mapped to plain-English messages, plus a lab seat-capacity warning.</t>
-  </si>
-  <si>
-    <t>Computer lab allocation</t>
-  </si>
-  <si>
-    <t>17 Aug 2026: already shipped — lab_id on timetable slots with capacity warning.</t>
-  </si>
-  <si>
-    <t>Link live session to timetable period</t>
-  </si>
-  <si>
-    <t>17 Aug 2026: live_sessions has no timetable_slot_id — sessions are not tied to a scheduled period.</t>
-  </si>
-  <si>
-    <t>Tue 18 Aug</t>
-  </si>
-  <si>
-    <t>Substitute teacher and rescheduling</t>
-  </si>
-  <si>
     <t>17 Aug 2026: rescheduling exists via timetable_exceptions. Substitute teacher not modelled.</t>
   </si>
   <si>
-    <t>Attendance recording</t>
-  </si>
-  <si>
-    <t>17 Aug 2026: session_participants records joins, but there is no attendance register or report.</t>
-  </si>
-  <si>
-    <t>Tablet usability fixes</t>
+    <t xml:space="preserve">bulk import </t>
   </si>
   <si>
     <t>5. Teacher</t>
   </si>
   <si>
-    <t>Exam builder - responsive form and validation</t>
-  </si>
-  <si>
-    <t>17 Aug 2026: server-side validation done; responsive pass not started.</t>
-  </si>
-  <si>
     <t>Exam publish - transactional and scope validation</t>
   </si>
   <si>
@@ -348,10 +339,13 @@
     <t>PIN login - roster search and duplicate names</t>
   </si>
   <si>
-    <t>Image based quizzes</t>
-  </si>
-  <si>
-    <t>Exam autosave, retry and offline indicator</t>
+    <t>Image based games</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exam </t>
+  </si>
+  <si>
+    <t>in progress</t>
   </si>
   <si>
     <t>Virtual lab UI improvements</t>
@@ -360,37 +354,31 @@
     <t>Fri 21 Aug</t>
   </si>
   <si>
-    <t>Exam submit confirmation and refresh recovery</t>
-  </si>
-  <si>
-    <t>Proper quizzes inside virtual labs</t>
+    <t xml:space="preserve">AI tutor - vision response </t>
   </si>
   <si>
     <t>AI chat - responsive and retry states</t>
   </si>
   <si>
-    <t>Today's Lab screen and period timer</t>
-  </si>
-  <si>
-    <t>Reconnect and shared computer handoff</t>
-  </si>
-  <si>
-    <t>Badges, streaks and challenge error states</t>
+    <t xml:space="preserve">Adding Redis to overall code </t>
+  </si>
+  <si>
+    <t>Badges, streaks and challenge error states- remove</t>
+  </si>
+  <si>
+    <t>done</t>
   </si>
   <si>
     <t>Sat 22 Aug</t>
   </si>
   <si>
-    <t>Reduced motion and low performance mode</t>
+    <t>UI changes</t>
   </si>
   <si>
     <t>7. Support Ticket</t>
   </si>
   <si>
-    <t>Ticket notifications</t>
-  </si>
-  <si>
-    <t>Attachment upload validation</t>
+    <t xml:space="preserve">only for school admin </t>
   </si>
   <si>
     <t>Role based ticket visibility</t>
@@ -604,7 +592,7 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -623,13 +611,6 @@
     <font>
       <b/>
       <sz val="11"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -1118,148 +1099,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1666,7 +1647,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F89"/>
+  <dimension ref="A1:F84"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -2071,10 +2052,10 @@
         <v>53</v>
       </c>
       <c r="E21" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F21" s="5" t="s">
         <v>54</v>
-      </c>
-      <c r="F21" s="5" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="22" ht="30" spans="1:6">
@@ -2088,18 +2069,18 @@
         <v>52</v>
       </c>
       <c r="D22" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="E22" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F22" s="5" t="s">
         <v>56</v>
-      </c>
-      <c r="E22" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="F22" s="5" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="23" s="2" customFormat="1" ht="18" customHeight="1" spans="1:6">
       <c r="A23" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B23" s="8"/>
       <c r="C23" s="8"/>
@@ -2109,22 +2090,22 @@
     </row>
     <row r="24" spans="1:6">
       <c r="A24" t="s">
+        <v>57</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>58</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>59</v>
       </c>
       <c r="C24" t="s">
         <v>52</v>
       </c>
       <c r="D24" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="E24" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F24" s="5" t="s">
         <v>60</v>
-      </c>
-      <c r="E24" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="F24" s="5" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -2138,10 +2119,10 @@
         <v>52</v>
       </c>
       <c r="D25" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="E25" s="11" t="s">
         <v>62</v>
-      </c>
-      <c r="E25" s="11" t="s">
-        <v>39</v>
       </c>
       <c r="F25" s="5" t="s">
         <v>63</v>
@@ -2161,7 +2142,7 @@
         <v>64</v>
       </c>
       <c r="E26" s="11" t="s">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="F26" s="5" t="s">
         <v>65</v>
@@ -2221,7 +2202,7 @@
         <v>71</v>
       </c>
       <c r="E29" s="11" t="s">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="F29" s="5" t="s">
         <v>72</v>
@@ -2229,7 +2210,7 @@
     </row>
     <row r="30" spans="1:6">
       <c r="A30" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>73</v>
@@ -2241,10 +2222,10 @@
         <v>74</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>54</v>
+        <v>75</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -2258,16 +2239,16 @@
         <v>66</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E31" s="11" t="s">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="32" ht="30" spans="1:6">
       <c r="A32" t="s">
         <v>13</v>
       </c>
@@ -2275,56 +2256,56 @@
         <v>13</v>
       </c>
       <c r="C32" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="D32" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E32" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F32" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="33" ht="30" spans="1:6">
+      <c r="A33" t="s">
+        <v>13</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C33" t="s">
         <v>78</v>
       </c>
-      <c r="E32" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="F32" s="5" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6">
-      <c r="A33" t="s">
-        <v>13</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C33" t="s">
-        <v>79</v>
-      </c>
       <c r="D33" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="E33" s="11" t="s">
-        <v>39</v>
+        <v>81</v>
+      </c>
+      <c r="E33" s="10" t="s">
+        <v>11</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="34" ht="30" spans="1:6">
       <c r="A34" t="s">
-        <v>13</v>
+        <v>57</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>13</v>
+        <v>83</v>
       </c>
       <c r="C34" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E34" s="10" t="s">
         <v>11</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="35" ht="30" spans="1:6">
@@ -2335,36 +2316,36 @@
         <v>13</v>
       </c>
       <c r="C35" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E35" s="10" t="s">
         <v>11</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="36" ht="30" spans="1:6">
       <c r="A36" t="s">
-        <v>58</v>
+        <v>13</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>86</v>
+        <v>13</v>
       </c>
       <c r="C36" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E36" s="10" t="s">
         <v>11</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="37" ht="30" spans="1:6">
@@ -2375,16 +2356,16 @@
         <v>13</v>
       </c>
       <c r="C37" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>11</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="38" ht="30" spans="1:6">
@@ -2395,19 +2376,19 @@
         <v>13</v>
       </c>
       <c r="C38" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E38" s="10" t="s">
         <v>11</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="39" ht="30" spans="1:6">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
       <c r="A39" t="s">
         <v>13</v>
       </c>
@@ -2415,36 +2396,36 @@
         <v>13</v>
       </c>
       <c r="C39" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="E39" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="E39" s="11" t="s">
         <v>11</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="40" ht="30" spans="1:6">
       <c r="A40" t="s">
-        <v>13</v>
+        <v>57</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>13</v>
+        <v>96</v>
       </c>
       <c r="C40" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="E40" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="E40" s="9" t="s">
         <v>11</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="41" spans="1:6">
@@ -2455,36 +2436,36 @@
         <v>13</v>
       </c>
       <c r="C41" t="s">
-        <v>79</v>
+        <v>99</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="42" ht="30" spans="1:6">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6">
       <c r="A42" t="s">
-        <v>58</v>
+        <v>13</v>
       </c>
       <c r="B42" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C42" t="s">
         <v>99</v>
       </c>
-      <c r="C42" t="s">
-        <v>79</v>
-      </c>
       <c r="D42" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="E42" s="9" t="s">
-        <v>54</v>
+        <v>101</v>
+      </c>
+      <c r="E42" s="11" t="s">
+        <v>11</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>101</v>
+        <v>13</v>
       </c>
     </row>
     <row r="43" spans="1:6">
@@ -2495,13 +2476,13 @@
         <v>13</v>
       </c>
       <c r="C43" t="s">
+        <v>99</v>
+      </c>
+      <c r="D43" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="D43" s="5" t="s">
-        <v>103</v>
-      </c>
       <c r="E43" s="11" t="s">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="F43" s="5" t="s">
         <v>13</v>
@@ -2515,13 +2496,13 @@
         <v>13</v>
       </c>
       <c r="C44" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D44" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="E44" s="11" t="s">
         <v>104</v>
-      </c>
-      <c r="E44" s="11" t="s">
-        <v>39</v>
       </c>
       <c r="F44" s="5" t="s">
         <v>13</v>
@@ -2535,13 +2516,13 @@
         <v>13</v>
       </c>
       <c r="C45" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D45" s="5" t="s">
         <v>105</v>
       </c>
       <c r="E45" s="11" t="s">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="F45" s="5" t="s">
         <v>13</v>
@@ -2549,19 +2530,19 @@
     </row>
     <row r="46" spans="1:6">
       <c r="A46" t="s">
-        <v>13</v>
+        <v>57</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>13</v>
+        <v>106</v>
       </c>
       <c r="C46" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E46" s="11" t="s">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="F46" s="5" t="s">
         <v>13</v>
@@ -2575,13 +2556,13 @@
         <v>13</v>
       </c>
       <c r="C47" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E47" s="11" t="s">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="F47" s="5" t="s">
         <v>13</v>
@@ -2589,19 +2570,19 @@
     </row>
     <row r="48" spans="1:6">
       <c r="A48" t="s">
-        <v>58</v>
+        <v>13</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>108</v>
+        <v>13</v>
       </c>
       <c r="C48" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D48" s="5" t="s">
         <v>109</v>
       </c>
       <c r="E48" s="11" t="s">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="F48" s="5" t="s">
         <v>13</v>
@@ -2615,13 +2596,13 @@
         <v>13</v>
       </c>
       <c r="C49" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D49" s="5" t="s">
         <v>110</v>
       </c>
       <c r="E49" s="11" t="s">
-        <v>39</v>
+        <v>111</v>
       </c>
       <c r="F49" s="5" t="s">
         <v>13</v>
@@ -2629,19 +2610,19 @@
     </row>
     <row r="50" spans="1:6">
       <c r="A50" t="s">
-        <v>13</v>
+        <v>57</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>13</v>
+        <v>112</v>
       </c>
       <c r="C50" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D50" s="5" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E50" s="11" t="s">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="F50" s="5" t="s">
         <v>13</v>
@@ -2655,13 +2636,13 @@
         <v>13</v>
       </c>
       <c r="C51" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="E51" s="11" t="s">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="F51" s="5" t="s">
         <v>13</v>
@@ -2675,13 +2656,13 @@
         <v>13</v>
       </c>
       <c r="C52" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="E52" s="11" t="s">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="F52" s="5" t="s">
         <v>13</v>
@@ -2695,13 +2676,13 @@
         <v>13</v>
       </c>
       <c r="C53" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="D53" s="5" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="E53" s="11" t="s">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="F53" s="5" t="s">
         <v>13</v>
@@ -2709,65 +2690,55 @@
     </row>
     <row r="54" spans="1:6">
       <c r="A54" t="s">
-        <v>58</v>
+        <v>13</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>115</v>
+        <v>13</v>
       </c>
       <c r="C54" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E54" s="11" t="s">
-        <v>39</v>
+        <v>104</v>
       </c>
       <c r="F54" s="5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="55" spans="1:6">
-      <c r="A55" t="s">
-        <v>13</v>
-      </c>
-      <c r="B55" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C55" t="s">
-        <v>117</v>
-      </c>
-      <c r="D55" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="E55" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="F55" s="5" t="s">
-        <v>13</v>
-      </c>
+    <row r="55" s="2" customFormat="1" ht="18" customHeight="1" spans="1:6">
+      <c r="A55" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="B55" s="8"/>
+      <c r="C55" s="8"/>
+      <c r="D55" s="8"/>
+      <c r="E55" s="8"/>
+      <c r="F55" s="8"/>
     </row>
     <row r="56" spans="1:6">
       <c r="A56" t="s">
-        <v>13</v>
+        <v>119</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>13</v>
+        <v>120</v>
       </c>
       <c r="C56" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="D56" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="E56" s="11" t="s">
-        <v>39</v>
+        <v>122</v>
+      </c>
+      <c r="E56" s="10" t="s">
+        <v>11</v>
       </c>
       <c r="F56" s="5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="57" ht="30" spans="1:6">
       <c r="A57" t="s">
         <v>13</v>
       </c>
@@ -2775,19 +2746,19 @@
         <v>13</v>
       </c>
       <c r="C57" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="D57" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="E57" s="11" t="s">
-        <v>39</v>
+        <v>124</v>
+      </c>
+      <c r="E57" s="10" t="s">
+        <v>11</v>
       </c>
       <c r="F57" s="5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="58" ht="30" spans="1:6">
       <c r="A58" t="s">
         <v>13</v>
       </c>
@@ -2795,16 +2766,16 @@
         <v>13</v>
       </c>
       <c r="C58" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="D58" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="E58" s="11" t="s">
-        <v>39</v>
+        <v>126</v>
+      </c>
+      <c r="E58" s="10" t="s">
+        <v>11</v>
       </c>
       <c r="F58" s="5" t="s">
-        <v>13</v>
+        <v>127</v>
       </c>
     </row>
     <row r="59" spans="1:6">
@@ -2815,69 +2786,79 @@
         <v>13</v>
       </c>
       <c r="C59" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="E59" s="11" t="s">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="F59" s="5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="60" s="2" customFormat="1" ht="18" customHeight="1" spans="1:6">
-      <c r="A60" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="B60" s="8"/>
-      <c r="C60" s="8"/>
-      <c r="D60" s="8"/>
-      <c r="E60" s="8"/>
-      <c r="F60" s="8"/>
-    </row>
-    <row r="61" spans="1:6">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="60" ht="30" spans="1:6">
+      <c r="A60" t="s">
+        <v>13</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C60" t="s">
+        <v>121</v>
+      </c>
+      <c r="D60" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E60" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F60" s="5" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="61" ht="30" spans="1:6">
       <c r="A61" t="s">
-        <v>123</v>
+        <v>13</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>124</v>
+        <v>13</v>
       </c>
       <c r="C61" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="E61" s="10" t="s">
-        <v>11</v>
+        <v>132</v>
+      </c>
+      <c r="E61" s="9" t="s">
+        <v>75</v>
       </c>
       <c r="F61" s="5" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="62" ht="30" spans="1:6">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="62" ht="45" spans="1:6">
       <c r="A62" t="s">
-        <v>13</v>
+        <v>119</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>13</v>
+        <v>134</v>
       </c>
       <c r="C62" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="E62" s="10" t="s">
-        <v>11</v>
+        <v>135</v>
+      </c>
+      <c r="E62" s="9" t="s">
+        <v>75</v>
       </c>
       <c r="F62" s="5" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="63" ht="30" spans="1:6">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6">
       <c r="A63" t="s">
         <v>13</v>
       </c>
@@ -2885,19 +2866,19 @@
         <v>13</v>
       </c>
       <c r="C63" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="E63" s="10" t="s">
-        <v>11</v>
+        <v>137</v>
+      </c>
+      <c r="E63" s="11" t="s">
+        <v>62</v>
       </c>
       <c r="F63" s="5" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="64" ht="45" spans="1:6">
       <c r="A64" t="s">
         <v>13</v>
       </c>
@@ -2905,19 +2886,19 @@
         <v>13</v>
       </c>
       <c r="C64" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="D64" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="E64" s="11" t="s">
-        <v>39</v>
+        <v>138</v>
+      </c>
+      <c r="E64" s="9" t="s">
+        <v>75</v>
       </c>
       <c r="F64" s="5" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="65" ht="30" spans="1:6">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6">
       <c r="A65" t="s">
         <v>13</v>
       </c>
@@ -2925,19 +2906,19 @@
         <v>13</v>
       </c>
       <c r="C65" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="D65" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="E65" s="10" t="s">
-        <v>11</v>
+        <v>140</v>
+      </c>
+      <c r="E65" s="11" t="s">
+        <v>62</v>
       </c>
       <c r="F65" s="5" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="66" ht="30" spans="1:6">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6">
       <c r="A66" t="s">
         <v>13</v>
       </c>
@@ -2945,59 +2926,59 @@
         <v>13</v>
       </c>
       <c r="C66" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="D66" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="E66" s="9" t="s">
-        <v>54</v>
+        <v>141</v>
+      </c>
+      <c r="E66" s="11" t="s">
+        <v>62</v>
       </c>
       <c r="F66" s="5" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="67" ht="45" spans="1:6">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6">
       <c r="A67" t="s">
-        <v>123</v>
+        <v>13</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>138</v>
+        <v>13</v>
       </c>
       <c r="C67" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="D67" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="E67" s="9" t="s">
-        <v>54</v>
+        <v>142</v>
+      </c>
+      <c r="E67" s="11" t="s">
+        <v>62</v>
       </c>
       <c r="F67" s="5" t="s">
-        <v>140</v>
+        <v>13</v>
       </c>
     </row>
     <row r="68" spans="1:6">
       <c r="A68" t="s">
-        <v>13</v>
+        <v>119</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>13</v>
+        <v>143</v>
       </c>
       <c r="C68" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="D68" s="5" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="E68" s="11" t="s">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="F68" s="5" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="69" ht="45" spans="1:6">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6">
       <c r="A69" t="s">
         <v>13</v>
       </c>
@@ -3005,16 +2986,16 @@
         <v>13</v>
       </c>
       <c r="C69" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="D69" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="E69" s="9" t="s">
-        <v>54</v>
+        <v>145</v>
+      </c>
+      <c r="E69" s="11" t="s">
+        <v>62</v>
       </c>
       <c r="F69" s="5" t="s">
-        <v>143</v>
+        <v>13</v>
       </c>
     </row>
     <row r="70" spans="1:6">
@@ -3025,16 +3006,16 @@
         <v>13</v>
       </c>
       <c r="C70" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="D70" s="5" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E70" s="11" t="s">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="F70" s="5" t="s">
-        <v>61</v>
+        <v>13</v>
       </c>
     </row>
     <row r="71" spans="1:6">
@@ -3045,13 +3026,13 @@
         <v>13</v>
       </c>
       <c r="C71" t="s">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="D71" s="5" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="E71" s="11" t="s">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="F71" s="5" t="s">
         <v>13</v>
@@ -3065,13 +3046,13 @@
         <v>13</v>
       </c>
       <c r="C72" t="s">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="D72" s="5" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="E72" s="11" t="s">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="F72" s="5" t="s">
         <v>13</v>
@@ -3079,19 +3060,19 @@
     </row>
     <row r="73" spans="1:6">
       <c r="A73" t="s">
-        <v>123</v>
+        <v>13</v>
       </c>
       <c r="B73" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C73" t="s">
         <v>147</v>
       </c>
-      <c r="C73" t="s">
-        <v>125</v>
-      </c>
       <c r="D73" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E73" s="11" t="s">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="F73" s="5" t="s">
         <v>13</v>
@@ -3099,22 +3080,22 @@
     </row>
     <row r="74" spans="1:6">
       <c r="A74" t="s">
-        <v>13</v>
+        <v>119</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>13</v>
+        <v>151</v>
       </c>
       <c r="C74" t="s">
-        <v>125</v>
+        <v>9</v>
       </c>
       <c r="D74" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="E74" s="11" t="s">
-        <v>39</v>
+        <v>152</v>
+      </c>
+      <c r="E74" s="10" t="s">
+        <v>11</v>
       </c>
       <c r="F74" s="5" t="s">
-        <v>13</v>
+        <v>153</v>
       </c>
     </row>
     <row r="75" spans="1:6">
@@ -3125,19 +3106,19 @@
         <v>13</v>
       </c>
       <c r="C75" t="s">
-        <v>125</v>
+        <v>29</v>
       </c>
       <c r="D75" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="E75" s="11" t="s">
-        <v>39</v>
+        <v>154</v>
+      </c>
+      <c r="E75" s="9" t="s">
+        <v>75</v>
       </c>
       <c r="F75" s="5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="76" ht="30" spans="1:6">
       <c r="A76" t="s">
         <v>13</v>
       </c>
@@ -3145,16 +3126,16 @@
         <v>13</v>
       </c>
       <c r="C76" t="s">
-        <v>151</v>
+        <v>52</v>
       </c>
       <c r="D76" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="E76" s="11" t="s">
-        <v>39</v>
+        <v>156</v>
+      </c>
+      <c r="E76" s="10" t="s">
+        <v>11</v>
       </c>
       <c r="F76" s="5" t="s">
-        <v>13</v>
+        <v>157</v>
       </c>
     </row>
     <row r="77" spans="1:6">
@@ -3165,16 +3146,16 @@
         <v>13</v>
       </c>
       <c r="C77" t="s">
-        <v>151</v>
+        <v>66</v>
       </c>
       <c r="D77" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="E77" s="11" t="s">
-        <v>39</v>
+        <v>158</v>
+      </c>
+      <c r="E77" s="9" t="s">
+        <v>75</v>
       </c>
       <c r="F77" s="5" t="s">
-        <v>13</v>
+        <v>159</v>
       </c>
     </row>
     <row r="78" spans="1:6">
@@ -3185,59 +3166,49 @@
         <v>13</v>
       </c>
       <c r="C78" t="s">
-        <v>151</v>
+        <v>78</v>
       </c>
       <c r="D78" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="E78" s="11" t="s">
-        <v>39</v>
+        <v>160</v>
+      </c>
+      <c r="E78" s="9" t="s">
+        <v>75</v>
       </c>
       <c r="F78" s="5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6">
-      <c r="A79" t="s">
-        <v>123</v>
-      </c>
-      <c r="B79" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="C79" t="s">
-        <v>9</v>
-      </c>
-      <c r="D79" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="E79" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="F79" s="5" t="s">
-        <v>157</v>
-      </c>
+        <v>161</v>
+      </c>
+    </row>
+    <row r="79" s="2" customFormat="1" ht="18" customHeight="1" spans="1:6">
+      <c r="A79" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="B79" s="8"/>
+      <c r="C79" s="8"/>
+      <c r="D79" s="8"/>
+      <c r="E79" s="8"/>
+      <c r="F79" s="8"/>
     </row>
     <row r="80" spans="1:6">
       <c r="A80" t="s">
-        <v>13</v>
+        <v>162</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>13</v>
+        <v>163</v>
       </c>
       <c r="C80" t="s">
-        <v>29</v>
+        <v>78</v>
       </c>
       <c r="D80" s="5" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="E80" s="9" t="s">
-        <v>54</v>
+        <v>75</v>
       </c>
       <c r="F80" s="5" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="81" ht="30" spans="1:6">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6">
       <c r="A81" t="s">
         <v>13</v>
       </c>
@@ -3245,16 +3216,16 @@
         <v>13</v>
       </c>
       <c r="C81" t="s">
-        <v>52</v>
+        <v>78</v>
       </c>
       <c r="D81" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="E81" s="10" t="s">
-        <v>11</v>
+        <v>166</v>
+      </c>
+      <c r="E81" s="11" t="s">
+        <v>62</v>
       </c>
       <c r="F81" s="5" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
     </row>
     <row r="82" spans="1:6">
@@ -3265,19 +3236,19 @@
         <v>13</v>
       </c>
       <c r="C82" t="s">
-        <v>66</v>
+        <v>114</v>
       </c>
       <c r="D82" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="E82" s="9" t="s">
-        <v>54</v>
+        <v>168</v>
+      </c>
+      <c r="E82" s="11" t="s">
+        <v>62</v>
       </c>
       <c r="F82" s="5" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="83" ht="30" spans="1:6">
       <c r="A83" t="s">
         <v>13</v>
       </c>
@@ -3285,138 +3256,48 @@
         <v>13</v>
       </c>
       <c r="C83" t="s">
-        <v>79</v>
+        <v>121</v>
       </c>
       <c r="D83" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="E83" s="9" t="s">
-        <v>54</v>
+        <v>169</v>
+      </c>
+      <c r="E83" s="10" t="s">
+        <v>11</v>
       </c>
       <c r="F83" s="5" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="84" s="2" customFormat="1" ht="18" customHeight="1" spans="1:6">
-      <c r="A84" s="8" t="s">
-        <v>166</v>
-      </c>
-      <c r="B84" s="8"/>
-      <c r="C84" s="8"/>
-      <c r="D84" s="8"/>
-      <c r="E84" s="8"/>
-      <c r="F84" s="8"/>
-    </row>
-    <row r="85" spans="1:6">
-      <c r="A85" t="s">
-        <v>166</v>
-      </c>
-      <c r="B85" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="C85" t="s">
-        <v>79</v>
-      </c>
-      <c r="D85" s="5" t="s">
-        <v>168</v>
-      </c>
-      <c r="E85" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="F85" s="5" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6">
-      <c r="A86" t="s">
-        <v>13</v>
-      </c>
-      <c r="B86" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C86" t="s">
-        <v>79</v>
-      </c>
-      <c r="D86" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="E86" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="F86" s="5" t="s">
+    </row>
+    <row r="84" spans="1:6">
+      <c r="A84" t="s">
+        <v>13</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C84" t="s">
+        <v>147</v>
+      </c>
+      <c r="D84" s="5" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="87" spans="1:6">
-      <c r="A87" t="s">
-        <v>13</v>
-      </c>
-      <c r="B87" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C87" t="s">
-        <v>117</v>
-      </c>
-      <c r="D87" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="E87" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="F87" s="5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="88" ht="30" spans="1:6">
-      <c r="A88" t="s">
-        <v>13</v>
-      </c>
-      <c r="B88" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C88" t="s">
-        <v>125</v>
-      </c>
-      <c r="D88" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="E88" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="F88" s="5" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6">
-      <c r="A89" t="s">
-        <v>13</v>
-      </c>
-      <c r="B89" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C89" t="s">
-        <v>151</v>
-      </c>
-      <c r="D89" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="E89" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="F89" s="5" t="s">
+      <c r="E84" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="F84" s="5" t="s">
         <v>13</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A2:F89" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A2:F84" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <mergeCells count="5">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A23:F23"/>
-    <mergeCell ref="A60:F60"/>
-    <mergeCell ref="A84:F84"/>
+    <mergeCell ref="A55:F55"/>
+    <mergeCell ref="A79:F79"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="1" orientation="portrait"/>
@@ -3444,25 +3325,25 @@
         <v>1</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>54</v>
+        <v>75</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -3488,12 +3369,12 @@
         <v>2</v>
       </c>
       <c r="H2" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B3">
         <v>6</v>
@@ -3514,12 +3395,12 @@
         <v>0</v>
       </c>
       <c r="H3" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="B4">
         <v>4</v>
@@ -3540,12 +3421,12 @@
         <v>0</v>
       </c>
       <c r="H4" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -3566,12 +3447,12 @@
         <v>0</v>
       </c>
       <c r="H5" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
     </row>
     <row r="6" s="2" customFormat="1" spans="1:8">
       <c r="A6" s="4" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="B6" s="4">
         <v>15</v>
@@ -3592,12 +3473,12 @@
         <v>2</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1" spans="1:8">
       <c r="A8" s="5" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>

</xml_diff>